<commit_message>
Melhoria na coleta e exports
</commit_message>
<xml_diff>
--- a/relatorio_rpv.xlsx
+++ b/relatorio_rpv.xlsx
@@ -10,7 +10,7 @@
     <sheet name="RPVs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'RPVs'!$A$1:$F$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'RPVs'!$A$1:$G$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -491,6 +491,7 @@
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
@@ -524,81 +525,92 @@
           <t>Nº RPV</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Coletado em</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>MARIA RAIMUNDA NUNES DE SOUZA</t>
+          <t>VALERIA MARIA DOS SANTOS</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>0508950-51.2026.4.05.0000</t>
+          <t>0532713-81.2026.4.05.0000</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>00037583920254058502</t>
+          <t>00547444820254058000</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>7ª VARA FEDERAL - SE</t>
+          <t>6ª VARA FEDERAL - AL</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr"/>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>RPV0-SE</t>
+          <t>RPV4417865-AL</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>23/09/2026 12:41:29</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>MARCIA APARECIDA DA COSTA SILVA</t>
+          <t>EDSON ALVES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>0473849-50.2026.4.05.0000</t>
+          <t>0530289-66.2026.4.05.0000</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>00486439220254058000</t>
+          <t>00578467820254058000</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>9ª VARA FEDERAL - AL</t>
-        </is>
-      </c>
-      <c r="E3" s="7" t="inlineStr">
-        <is>
-          <t>CEF</t>
-        </is>
-      </c>
+          <t>6ª VARA FEDERAL - AL</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr"/>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>RPV4362512-AL</t>
+          <t>RPV4415557-AL</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>23/09/2026 12:41:29</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>MARIA VITORIA ALVES TORRES</t>
+          <t>JONATHAN LEVI GERONIMO DE SOUZA</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>0508729-68.2026.4.05.0000</t>
+          <t>0530253-24.2026.4.05.0000</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>00631730420254058000</t>
+          <t>00049087220264058000</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -609,232 +621,248 @@
       <c r="E4" s="4" t="inlineStr"/>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>RPV0-AL</t>
+          <t>RPV4415521-AL</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>23/09/2026 12:41:29</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>ANTONIO MARQUES DIAS</t>
+          <t>MARIA ANGELA DA SILVA SOUZA</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>0472988-64.2026.4.05.0000</t>
+          <t>0532701-67.2026.4.05.0000</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>00255725720224058100</t>
+          <t>00645605420254058000</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>14ª VARA FEDERAL - CE</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>CEF</t>
-        </is>
-      </c>
+          <t>6ª VARA FEDERAL - AL</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr"/>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>RPV4361679-CE</t>
+          <t>RPV4417853-AL</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>23/09/2026 12:41:29</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>ANTONIO MARQUES DIAS</t>
+          <t>AMARO NASCIMENTO DA SILVA</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>0472989-49.2026.4.05.0000</t>
+          <t>0532750-11.2026.4.05.0000</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>00255725720224058100</t>
+          <t>00035166420228172570</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>14ª VARA FEDERAL - CE</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>CEF</t>
-        </is>
-      </c>
+          <t>2ª Vara da Comarca de Escada - PE</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr"/>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>RPV4361680-CE</t>
+          <t>RPV4417902-PE</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>23/09/2026 12:41:29</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>GEDALVA COUTO FERNANDES</t>
+          <t>JOAO PEREIRA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>0508321-77.2026.4.05.0000</t>
+          <t>0532386-39.2026.4.05.0000</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>00019251720104058500</t>
+          <t>00005854620254058101</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>1ª VARA FEDERAL - SE</t>
+          <t>29ª VARA FEDERAL - CE</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr"/>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>RPV4394133-SE</t>
+          <t>RPV4417543-CE</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>23/09/2026 12:41:29</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>LUCIANA MARIA DOS SANTOS</t>
+          <t>JOELMA VALDECI DA SILVA</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>0473876-33.2026.4.05.0000</t>
+          <t>0531265-73.2026.4.05.0000</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>00189730920254058000</t>
+          <t>00369776720254058300</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>9ª VARA FEDERAL - AL</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>CEF</t>
-        </is>
-      </c>
+          <t>15ª VARA FEDERAL - PE</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr"/>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>RPV4362539-AL</t>
+          <t>RPV4416488-PE</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>23/09/2026 12:41:29</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>HELDER ROCHA FALCAO</t>
+          <t>AIRTON LIMA NORONHA JUNIOR</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>0475186-74.2026.4.05.0000</t>
+          <t>0528734-14.2026.4.05.0000</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>00051685520084058300</t>
+          <t>00005640320264058500</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>2ª VARA FEDERAL - PE</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>CEF</t>
-        </is>
-      </c>
+          <t>4ª VARA FEDERAL - SE</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr"/>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>RPV4363843-PE</t>
+          <t>RPV4414020-SE</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>23/09/2026 12:41:29</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>FERNANDO ANTONIO MENDES FACANHA FILHO</t>
+          <t>FILIPE DE JESUS PASSOS</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>0475581-66.2026.4.05.0000</t>
+          <t>0529967-46.2026.4.05.0000</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>00671075820254058100</t>
+          <t>00008516320264058500</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>33ª VARA FEDERAL - CE</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>CEF</t>
-        </is>
-      </c>
+          <t>4ª VARA FEDERAL - SE</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr"/>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>RPV4364217-CE</t>
+          <t>RPV4415236-SE</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>23/09/2026 12:41:29</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>LUCIENE DE ALMEIDA VIEIRA</t>
+          <t>CLAUDIA DA SILVA MELLO</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>0473889-32.2026.4.05.0000</t>
+          <t>0530355-46.2026.4.05.0000</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>00576025220254058000</t>
+          <t>00485209420254058000</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>9ª VARA FEDERAL - AL</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>CEF</t>
-        </is>
-      </c>
+          <t>6ª VARA FEDERAL - AL</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr"/>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>RPV4362552-AL</t>
+          <t>RPV4415623-AL</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>23/09/2026 12:41:29</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F11"/>
+  <autoFilter ref="A1:G11"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>

</xml_diff>